<commit_message>
feat(importer): GSA agency-bureau-property key, skip Disposed, legacy identity
Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01UbGohWWFx8ZBHApJgkMWrW
</commit_message>
<xml_diff>
--- a/importer/tests/fixtures/gsa_frpp_sample.xlsx
+++ b/importer/tests/fixtures/gsa_frpp_sample.xlsx
@@ -7,7 +7,7 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="sheet1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Sheet" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J9"/>
+  <dimension ref="A1:M15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -467,6 +467,21 @@
           <t>Installation Name</t>
         </is>
       </c>
+      <c r="K1" t="inlineStr">
+        <is>
+          <t>Reporting Agency Code</t>
+        </is>
+      </c>
+      <c r="L1" t="inlineStr">
+        <is>
+          <t>Reporting Bureau Code</t>
+        </is>
+      </c>
+      <c r="M1" t="inlineStr">
+        <is>
+          <t>Asset Status</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -515,6 +530,21 @@
           <t>Federal Office Building</t>
         </is>
       </c>
+      <c r="K2" t="inlineStr">
+        <is>
+          <t>47</t>
+        </is>
+      </c>
+      <c r="L2" t="inlineStr">
+        <is>
+          <t>00</t>
+        </is>
+      </c>
+      <c r="M2" t="inlineStr">
+        <is>
+          <t>Current Mission Need</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -557,6 +587,21 @@
           <t>US Courthouse Houston</t>
         </is>
       </c>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t>47</t>
+        </is>
+      </c>
+      <c r="L3" t="inlineStr">
+        <is>
+          <t>00</t>
+        </is>
+      </c>
+      <c r="M3" t="inlineStr">
+        <is>
+          <t>Current Mission Need</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -605,6 +650,21 @@
           <t>SF Federal Building</t>
         </is>
       </c>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>47</t>
+        </is>
+      </c>
+      <c r="L4" t="inlineStr">
+        <is>
+          <t>00</t>
+        </is>
+      </c>
+      <c r="M4" t="inlineStr">
+        <is>
+          <t>Current Mission Need</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -647,6 +707,21 @@
           <t>Vacant Federal Land</t>
         </is>
       </c>
+      <c r="K5" t="inlineStr">
+        <is>
+          <t>47</t>
+        </is>
+      </c>
+      <c r="L5" t="inlineStr">
+        <is>
+          <t>00</t>
+        </is>
+      </c>
+      <c r="M5" t="inlineStr">
+        <is>
+          <t>Current Mission Need</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -684,6 +759,21 @@
           <t>No Address Building</t>
         </is>
       </c>
+      <c r="K6" t="inlineStr">
+        <is>
+          <t>47</t>
+        </is>
+      </c>
+      <c r="L6" t="inlineStr">
+        <is>
+          <t>00</t>
+        </is>
+      </c>
+      <c r="M6" t="inlineStr">
+        <is>
+          <t>Current Mission Need</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -732,6 +822,21 @@
           <t>Mislocated Federal Building</t>
         </is>
       </c>
+      <c r="K7" t="inlineStr">
+        <is>
+          <t>47</t>
+        </is>
+      </c>
+      <c r="L7" t="inlineStr">
+        <is>
+          <t>00</t>
+        </is>
+      </c>
+      <c r="M7" t="inlineStr">
+        <is>
+          <t>Current Mission Need</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -780,6 +885,21 @@
           <t>DALLAS, TX</t>
         </is>
       </c>
+      <c r="K8" t="inlineStr">
+        <is>
+          <t>47</t>
+        </is>
+      </c>
+      <c r="L8" t="inlineStr">
+        <is>
+          <t>00</t>
+        </is>
+      </c>
+      <c r="M8" t="inlineStr">
+        <is>
+          <t>Current Mission Need</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -826,6 +946,382 @@
       <c r="J9" t="inlineStr">
         <is>
           <t>1234 Main Street</t>
+        </is>
+      </c>
+      <c r="K9" t="inlineStr">
+        <is>
+          <t>47</t>
+        </is>
+      </c>
+      <c r="L9" t="inlineStr">
+        <is>
+          <t>00</t>
+        </is>
+      </c>
+      <c r="M9" t="inlineStr">
+        <is>
+          <t>Current Mission Need</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>RPUID-TX-DUP</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Building</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>Office</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>10 Alamo Plaza</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>San Antonio</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>TEXAS</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>78205</t>
+        </is>
+      </c>
+      <c r="H10" t="n">
+        <v>29.4241</v>
+      </c>
+      <c r="I10" t="n">
+        <v>-98.4936</v>
+      </c>
+      <c r="J10" t="inlineStr">
+        <is>
+          <t>San Antonio Federal Center</t>
+        </is>
+      </c>
+      <c r="K10" t="inlineStr">
+        <is>
+          <t>13</t>
+        </is>
+      </c>
+      <c r="L10" t="inlineStr">
+        <is>
+          <t>14</t>
+        </is>
+      </c>
+      <c r="M10" t="inlineStr">
+        <is>
+          <t>Current Mission Need</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>RPUID-TX-DUP</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Building</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>Office</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>20 Broadway</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>Lubbock</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>TEXAS</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>79401</t>
+        </is>
+      </c>
+      <c r="H11" t="n">
+        <v>33.5779</v>
+      </c>
+      <c r="I11" t="n">
+        <v>-101.8552</v>
+      </c>
+      <c r="J11" t="inlineStr">
+        <is>
+          <t>Lubbock Federal Building</t>
+        </is>
+      </c>
+      <c r="K11" t="inlineStr">
+        <is>
+          <t>14</t>
+        </is>
+      </c>
+      <c r="L11" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="M11" t="inlineStr">
+        <is>
+          <t>Determination to Dispose</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>RPUID-TX-GONE</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Building</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>Office</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>30 Austin Ave</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>Waco</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>TEXAS</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>76701</t>
+        </is>
+      </c>
+      <c r="H12" t="n">
+        <v>31.5493</v>
+      </c>
+      <c r="I12" t="n">
+        <v>-97.1467</v>
+      </c>
+      <c r="J12" t="inlineStr">
+        <is>
+          <t>Former Federal Building</t>
+        </is>
+      </c>
+      <c r="K12" t="inlineStr">
+        <is>
+          <t>47</t>
+        </is>
+      </c>
+      <c r="L12" t="inlineStr">
+        <is>
+          <t>00</t>
+        </is>
+      </c>
+      <c r="M12" t="inlineStr">
+        <is>
+          <t>Disposed</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>RPUID-TX-NOBUREAU</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Building</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>Office</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>40 Broadway</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>Tyler</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>TEXAS</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>75701</t>
+        </is>
+      </c>
+      <c r="H13" t="n">
+        <v>32.3513</v>
+      </c>
+      <c r="I13" t="n">
+        <v>-95.30110000000001</v>
+      </c>
+      <c r="J13" t="inlineStr">
+        <is>
+          <t>Tyler Federal Building</t>
+        </is>
+      </c>
+      <c r="K13" t="inlineStr">
+        <is>
+          <t>47</t>
+        </is>
+      </c>
+      <c r="M13" t="inlineStr">
+        <is>
+          <t>Current Mission Need</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>RPUID-TX-GEO</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>Building</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>Office</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>50 Smith St</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>Houston</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>TEXAS</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>77002</t>
+        </is>
+      </c>
+      <c r="J14" t="inlineStr">
+        <is>
+          <t>Houston Annex A</t>
+        </is>
+      </c>
+      <c r="K14" t="inlineStr">
+        <is>
+          <t>13</t>
+        </is>
+      </c>
+      <c r="L14" t="inlineStr">
+        <is>
+          <t>14</t>
+        </is>
+      </c>
+      <c r="M14" t="inlineStr">
+        <is>
+          <t>Current Mission Need</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>RPUID-TX-GEO</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>Building</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>Office</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>60 Fannin St</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>Houston</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>TEXAS</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>77002</t>
+        </is>
+      </c>
+      <c r="J15" t="inlineStr">
+        <is>
+          <t>Houston Annex B</t>
+        </is>
+      </c>
+      <c r="K15" t="inlineStr">
+        <is>
+          <t>14</t>
+        </is>
+      </c>
+      <c r="L15" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="M15" t="inlineStr">
+        <is>
+          <t>Current Mission Need</t>
         </is>
       </c>
     </row>

</xml_diff>